<commit_message>
feat: enhance parseValue function to support various number formats and improve data parsing
</commit_message>
<xml_diff>
--- a/importacao/faturasdetalhes.xlsx
+++ b/importacao/faturasdetalhes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edson\Documents\GitHub\acordus\importacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C0F4FD9-AF51-47EE-BCDA-AEA5D7282A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4598158-4FD5-4713-BAD1-DA125FC5D85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -660,6 +663,13 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -714,10 +724,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -737,20 +748,25 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1059,22 +1075,22 @@
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.140625" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1093,52 +1109,52 @@
       <c r="E1" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>128</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="7" t="s">
         <v>130</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="7" t="s">
         <v>132</v>
       </c>
       <c r="K1" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="7" t="s">
         <v>134</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="7" t="s">
         <v>136</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>138</v>
       </c>
       <c r="Q1" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="7" t="s">
         <v>140</v>
       </c>
       <c r="S1" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="11" t="s">
         <v>143</v>
       </c>
     </row>
@@ -1191,7 +1207,7 @@
       <c r="P2" s="8">
         <v>-42.88</v>
       </c>
-      <c r="U2" s="9">
+      <c r="U2" s="12">
         <v>1171.8</v>
       </c>
     </row>
@@ -1211,46 +1227,46 @@
       <c r="E3" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="9">
         <v>850</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J3" s="9">
         <v>50</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="9">
         <v>70</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N3" s="10">
+      <c r="N3" s="9">
         <v>37</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="P3" s="10">
+      <c r="P3" s="9">
         <v>170</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="R3" s="10">
+      <c r="R3" s="9">
         <v>141</v>
       </c>
-      <c r="U3" s="9">
+      <c r="U3" s="12">
         <v>1357.8</v>
       </c>
     </row>
@@ -1309,7 +1325,7 @@
       <c r="R4" s="8">
         <v>170</v>
       </c>
-      <c r="U4" s="9">
+      <c r="U4" s="12">
         <v>1357.8</v>
       </c>
     </row>
@@ -1329,46 +1345,46 @@
       <c r="E5" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <v>900</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="9">
         <v>50</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L5" s="9">
         <v>70</v>
       </c>
       <c r="M5" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N5" s="10">
+      <c r="N5" s="9">
         <v>37</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P5" s="10">
+      <c r="P5" s="9">
         <v>85</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="R5" s="10">
-        <v>150</v>
-      </c>
-      <c r="U5" s="9">
+      <c r="R5" s="9">
+        <v>150</v>
+      </c>
+      <c r="U5" s="12">
         <v>1331.8</v>
       </c>
     </row>
@@ -1427,7 +1443,7 @@
       <c r="R6" s="8">
         <v>158</v>
       </c>
-      <c r="U6" s="9">
+      <c r="U6" s="12">
         <v>1474.8</v>
       </c>
     </row>
@@ -1447,34 +1463,34 @@
       <c r="E7" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="9">
         <v>700</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="9">
         <v>85</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="9">
         <v>37</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L7" s="10">
+      <c r="L7" s="9">
         <v>70</v>
       </c>
       <c r="M7" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N7" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U7" s="9">
+      <c r="N7" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U7" s="12">
         <v>931.8</v>
       </c>
     </row>
@@ -1533,7 +1549,7 @@
       <c r="R8" s="8">
         <v>100</v>
       </c>
-      <c r="U8" s="9">
+      <c r="U8" s="12">
         <v>979</v>
       </c>
     </row>
@@ -1553,40 +1569,40 @@
       <c r="E9" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="9">
         <v>850</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="9">
         <v>50</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="9">
         <v>37</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="L9" s="10">
+      <c r="L9" s="9">
         <v>85</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N9" s="10">
+      <c r="N9" s="9">
         <v>70</v>
       </c>
       <c r="O9" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="P9" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U9" s="9">
+      <c r="P9" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U9" s="12">
         <v>1131.8</v>
       </c>
     </row>
@@ -1645,7 +1661,7 @@
       <c r="R10" s="8">
         <v>141</v>
       </c>
-      <c r="U10" s="9">
+      <c r="U10" s="12">
         <v>1357.8</v>
       </c>
     </row>
@@ -1665,46 +1681,46 @@
       <c r="E11" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="9">
         <v>700</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="9">
         <v>50</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="9">
         <v>37</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="M11" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N11" s="10">
+      <c r="N11" s="9">
         <v>70</v>
       </c>
       <c r="O11" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P11" s="10">
+      <c r="P11" s="9">
         <v>85</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="R11" s="10">
+      <c r="R11" s="9">
         <v>116</v>
       </c>
-      <c r="U11" s="9">
+      <c r="U11" s="12">
         <v>1097.8</v>
       </c>
     </row>
@@ -1763,7 +1779,7 @@
       <c r="R12" s="8">
         <v>-37</v>
       </c>
-      <c r="U12" s="9">
+      <c r="U12" s="12">
         <v>1095.07</v>
       </c>
     </row>
@@ -1783,40 +1799,40 @@
       <c r="E13" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="9">
         <v>700</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="9">
         <v>85</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="J13" s="10">
+      <c r="J13" s="9">
         <v>37</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L13" s="10">
+      <c r="L13" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="N13" s="10">
+      <c r="N13" s="9">
         <v>50</v>
       </c>
       <c r="O13" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="P13" s="10">
+      <c r="P13" s="9">
         <v>50</v>
       </c>
-      <c r="U13" s="9">
+      <c r="U13" s="12">
         <v>961.8</v>
       </c>
     </row>
@@ -1875,7 +1891,7 @@
       <c r="R14" s="8">
         <v>-95</v>
       </c>
-      <c r="U14" s="9">
+      <c r="U14" s="12">
         <v>931.8</v>
       </c>
     </row>
@@ -1895,46 +1911,46 @@
       <c r="E15" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="9">
         <v>850</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="9">
         <v>170</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J15" s="10">
+      <c r="J15" s="9">
         <v>37</v>
       </c>
       <c r="K15" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="L15" s="10">
+      <c r="L15" s="9">
         <v>50</v>
       </c>
       <c r="M15" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N15" s="10">
+      <c r="N15" s="9">
         <v>70</v>
       </c>
       <c r="O15" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="P15" s="10">
+      <c r="P15" s="9">
         <v>110</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="R15" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U15" s="9">
+      <c r="R15" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U15" s="12">
         <v>1326.8</v>
       </c>
     </row>
@@ -1993,7 +2009,7 @@
       <c r="R16" s="8">
         <v>85</v>
       </c>
-      <c r="U16" s="9">
+      <c r="U16" s="12">
         <v>981.8</v>
       </c>
     </row>
@@ -2013,40 +2029,40 @@
       <c r="E17" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="9">
         <v>678.87</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="9">
         <v>60</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J17" s="10">
+      <c r="J17" s="9">
         <v>37</v>
       </c>
       <c r="K17" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="L17" s="10">
+      <c r="L17" s="9">
         <v>170</v>
       </c>
       <c r="M17" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N17" s="10">
+      <c r="N17" s="9">
         <v>70</v>
       </c>
       <c r="O17" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="P17" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U17" s="9">
+      <c r="P17" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U17" s="12">
         <v>1055.67</v>
       </c>
     </row>
@@ -2111,7 +2127,7 @@
       <c r="T18" s="8">
         <v>100</v>
       </c>
-      <c r="U18" s="9">
+      <c r="U18" s="12">
         <v>1457.8</v>
       </c>
     </row>
@@ -2131,46 +2147,46 @@
       <c r="E19" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="9">
         <v>600</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J19" s="10">
+      <c r="J19" s="9">
         <v>50</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L19" s="10">
+      <c r="L19" s="9">
         <v>70</v>
       </c>
       <c r="M19" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N19" s="10">
+      <c r="N19" s="9">
         <v>37</v>
       </c>
       <c r="O19" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="P19" s="10">
+      <c r="P19" s="9">
         <v>100</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="R19" s="10">
+      <c r="R19" s="9">
         <v>85</v>
       </c>
-      <c r="U19" s="9">
+      <c r="U19" s="12">
         <v>981.8</v>
       </c>
     </row>
@@ -2229,7 +2245,7 @@
       <c r="R20" s="8">
         <v>-50</v>
       </c>
-      <c r="U20" s="9">
+      <c r="U20" s="12">
         <v>881.8</v>
       </c>
     </row>
@@ -2249,52 +2265,52 @@
       <c r="E21" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="9">
         <v>850</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J21" s="10">
+      <c r="J21" s="9">
         <v>50</v>
       </c>
       <c r="K21" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L21" s="10">
+      <c r="L21" s="9">
         <v>70</v>
       </c>
       <c r="M21" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N21" s="10">
+      <c r="N21" s="9">
         <v>37</v>
       </c>
       <c r="O21" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="P21" s="10">
+      <c r="P21" s="9">
         <v>141</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="R21" s="10">
+      <c r="R21" s="9">
         <v>85</v>
       </c>
       <c r="S21" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="T21" s="10">
+      <c r="T21" s="9">
         <v>5</v>
       </c>
-      <c r="U21" s="9">
+      <c r="U21" s="12">
         <v>1277.8</v>
       </c>
     </row>
@@ -2353,7 +2369,7 @@
       <c r="R22" s="8">
         <v>85</v>
       </c>
-      <c r="U22" s="9">
+      <c r="U22" s="12">
         <v>1272.8</v>
       </c>
     </row>
@@ -2373,46 +2389,46 @@
       <c r="E23" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="9">
         <v>1100</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="9">
         <v>50</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J23" s="10">
+      <c r="J23" s="9">
         <v>37</v>
       </c>
       <c r="K23" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L23" s="10">
+      <c r="L23" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="M23" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N23" s="10">
+      <c r="N23" s="9">
         <v>70</v>
       </c>
       <c r="O23" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="P23" s="10">
+      <c r="P23" s="9">
         <v>170</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="R23" s="10">
+      <c r="R23" s="9">
         <v>183</v>
       </c>
-      <c r="U23" s="9">
+      <c r="U23" s="12">
         <v>1649.8</v>
       </c>
     </row>
@@ -2465,7 +2481,7 @@
       <c r="P24" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U24" s="9">
+      <c r="U24" s="12">
         <v>1131.8</v>
       </c>
     </row>
@@ -2485,34 +2501,34 @@
       <c r="E25" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F25" s="9">
         <v>850</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="9">
         <v>70</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J25" s="9">
         <v>37</v>
       </c>
       <c r="K25" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="L25" s="10">
+      <c r="L25" s="9">
         <v>170</v>
       </c>
       <c r="M25" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N25" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U25" s="9">
+      <c r="N25" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U25" s="12">
         <v>1166.8</v>
       </c>
     </row>
@@ -2577,7 +2593,7 @@
       <c r="T26" s="8">
         <v>305</v>
       </c>
-      <c r="U26" s="9">
+      <c r="U26" s="12">
         <v>1577.8</v>
       </c>
     </row>
@@ -2597,34 +2613,34 @@
       <c r="E27" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F27" s="10">
+      <c r="F27" s="9">
         <v>680.43</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="9">
         <v>170</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="J27" s="10">
+      <c r="J27" s="9">
         <v>37</v>
       </c>
       <c r="K27" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="L27" s="10">
+      <c r="L27" s="9">
         <v>70</v>
       </c>
       <c r="M27" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N27" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U27" s="9">
+      <c r="N27" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U27" s="12">
         <v>997.23</v>
       </c>
     </row>
@@ -2671,7 +2687,7 @@
       <c r="N28" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U28" s="9">
+      <c r="U28" s="12">
         <v>1321.8</v>
       </c>
     </row>
@@ -2691,40 +2707,40 @@
       <c r="E29" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F29" s="10">
+      <c r="F29" s="9">
         <v>684.78</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H29" s="9">
         <v>85</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J29" s="10">
+      <c r="J29" s="9">
         <v>37</v>
       </c>
       <c r="K29" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L29" s="10">
+      <c r="L29" s="9">
         <v>70</v>
       </c>
       <c r="M29" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N29" s="10">
+      <c r="N29" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="O29" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="P29" s="10">
+      <c r="P29" s="9">
         <v>166</v>
       </c>
-      <c r="U29" s="9">
+      <c r="U29" s="12">
         <v>1082.58</v>
       </c>
     </row>
@@ -2783,7 +2799,7 @@
       <c r="R30" s="8">
         <v>85</v>
       </c>
-      <c r="U30" s="9">
+      <c r="U30" s="12">
         <v>1272.8</v>
       </c>
     </row>
@@ -2803,34 +2819,34 @@
       <c r="E31" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F31" s="10">
+      <c r="F31" s="9">
         <v>810</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="10">
+      <c r="H31" s="9">
         <v>85</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J31" s="10">
+      <c r="J31" s="9">
         <v>37</v>
       </c>
       <c r="K31" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="L31" s="10">
+      <c r="L31" s="9">
         <v>110</v>
       </c>
       <c r="M31" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N31" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U31" s="9">
+      <c r="N31" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U31" s="12">
         <v>1081.8</v>
       </c>
     </row>
@@ -2883,7 +2899,7 @@
       <c r="P32" s="8">
         <v>50</v>
       </c>
-      <c r="U32" s="9">
+      <c r="U32" s="12">
         <v>1129</v>
       </c>
     </row>
@@ -2903,46 +2919,46 @@
       <c r="E33" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F33" s="10">
+      <c r="F33" s="9">
         <v>679</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H33" s="10">
+      <c r="H33" s="9">
         <v>85</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="J33" s="10">
+      <c r="J33" s="9">
         <v>70</v>
       </c>
       <c r="K33" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="L33" s="10">
+      <c r="L33" s="9">
         <v>37</v>
       </c>
       <c r="M33" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="N33" s="10">
+      <c r="N33" s="9">
         <v>60</v>
       </c>
       <c r="O33" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="P33" s="10">
+      <c r="P33" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="R33" s="10">
+      <c r="R33" s="9">
         <v>-58</v>
       </c>
-      <c r="U33" s="9">
+      <c r="U33" s="12">
         <v>912.8</v>
       </c>
     </row>
@@ -2995,7 +3011,7 @@
       <c r="P34" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U34" s="9">
+      <c r="U34" s="12">
         <v>1131.8</v>
       </c>
     </row>
@@ -3015,34 +3031,34 @@
       <c r="E35" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F35" s="10">
+      <c r="F35" s="9">
         <v>683.35</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="H35" s="10">
+      <c r="H35" s="9">
         <v>37</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="J35" s="10">
+      <c r="J35" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="K35" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="L35" s="10">
+      <c r="L35" s="9">
         <v>170</v>
       </c>
       <c r="M35" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="N35" s="10">
+      <c r="N35" s="9">
         <v>60</v>
       </c>
-      <c r="U35" s="9">
+      <c r="U35" s="12">
         <v>990.15</v>
       </c>
     </row>
@@ -3089,7 +3105,7 @@
       <c r="N36" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U36" s="9">
+      <c r="U36" s="12">
         <v>925.08</v>
       </c>
     </row>
@@ -3109,46 +3125,46 @@
       <c r="E37" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F37" s="10">
+      <c r="F37" s="9">
         <v>850</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H37" s="10">
+      <c r="H37" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J37" s="10">
+      <c r="J37" s="9">
         <v>50</v>
       </c>
       <c r="K37" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L37" s="10">
+      <c r="L37" s="9">
         <v>70</v>
       </c>
       <c r="M37" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N37" s="10">
+      <c r="N37" s="9">
         <v>37</v>
       </c>
       <c r="O37" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="P37" s="10">
+      <c r="P37" s="9">
         <v>141</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="R37" s="10">
+      <c r="R37" s="9">
         <v>170</v>
       </c>
-      <c r="U37" s="9">
+      <c r="U37" s="12">
         <v>1357.8</v>
       </c>
     </row>
@@ -3195,7 +3211,7 @@
       <c r="N38" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U38" s="9">
+      <c r="U38" s="12">
         <v>1146.8</v>
       </c>
     </row>
@@ -3215,52 +3231,52 @@
       <c r="E39" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F39" s="10">
+      <c r="F39" s="9">
         <v>850</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H39" s="10">
+      <c r="H39" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J39" s="10">
+      <c r="J39" s="9">
         <v>50</v>
       </c>
       <c r="K39" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L39" s="10">
+      <c r="L39" s="9">
         <v>70</v>
       </c>
       <c r="M39" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N39" s="10">
+      <c r="N39" s="9">
         <v>37</v>
       </c>
       <c r="O39" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="P39" s="10">
+      <c r="P39" s="9">
         <v>170</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="R39" s="10">
+      <c r="R39" s="9">
         <v>141</v>
       </c>
       <c r="S39" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="T39" s="10">
+      <c r="T39" s="9">
         <v>60</v>
       </c>
-      <c r="U39" s="9">
+      <c r="U39" s="12">
         <v>1417.8</v>
       </c>
     </row>
@@ -3313,7 +3329,7 @@
       <c r="P40" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U40" s="9">
+      <c r="U40" s="12">
         <v>1216.8</v>
       </c>
     </row>
@@ -3333,34 +3349,34 @@
       <c r="E41" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F41" s="10">
+      <c r="F41" s="9">
         <v>850</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="H41" s="10">
+      <c r="H41" s="9">
         <v>85</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J41" s="10">
+      <c r="J41" s="9">
         <v>50</v>
       </c>
       <c r="K41" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="L41" s="10">
+      <c r="L41" s="9">
         <v>37</v>
       </c>
       <c r="M41" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N41" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U41" s="9">
+      <c r="N41" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U41" s="12">
         <v>1061.8</v>
       </c>
     </row>
@@ -3413,7 +3429,7 @@
       <c r="P42" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U42" s="9">
+      <c r="U42" s="12">
         <v>1381.8</v>
       </c>
     </row>
@@ -3433,40 +3449,40 @@
       <c r="E43" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F43" s="10">
+      <c r="F43" s="9">
         <v>695.67</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="H43" s="10">
+      <c r="H43" s="9">
         <v>85</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J43" s="10">
+      <c r="J43" s="9">
         <v>37</v>
       </c>
       <c r="K43" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L43" s="10">
+      <c r="L43" s="9">
         <v>70</v>
       </c>
       <c r="M43" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N43" s="10">
+      <c r="N43" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="O43" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="P43" s="10">
+      <c r="P43" s="9">
         <v>-45</v>
       </c>
-      <c r="U43" s="9">
+      <c r="U43" s="12">
         <v>882.47</v>
       </c>
     </row>
@@ -3519,7 +3535,7 @@
       <c r="P44" s="8">
         <v>-45</v>
       </c>
-      <c r="U44" s="9">
+      <c r="U44" s="12">
         <v>882.47</v>
       </c>
     </row>
@@ -3539,40 +3555,40 @@
       <c r="E45" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F45" s="10">
+      <c r="F45" s="9">
         <v>600</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H45" s="10">
+      <c r="H45" s="9">
         <v>50</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J45" s="10">
+      <c r="J45" s="9">
         <v>37</v>
       </c>
       <c r="K45" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L45" s="10">
+      <c r="L45" s="9">
         <v>37</v>
       </c>
       <c r="M45" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N45" s="10">
+      <c r="N45" s="9">
         <v>70</v>
       </c>
       <c r="O45" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P45" s="10">
+      <c r="P45" s="9">
         <v>85</v>
       </c>
-      <c r="U45" s="9">
+      <c r="U45" s="12">
         <v>879</v>
       </c>
     </row>
@@ -3625,7 +3641,7 @@
       <c r="P46" s="8">
         <v>85</v>
       </c>
-      <c r="U46" s="9">
+      <c r="U46" s="12">
         <v>879</v>
       </c>
     </row>
@@ -3645,34 +3661,34 @@
       <c r="E47" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F47" s="10">
+      <c r="F47" s="9">
         <v>700</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H47" s="10">
+      <c r="H47" s="9">
         <v>85</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="J47" s="10">
+      <c r="J47" s="9">
         <v>37</v>
       </c>
       <c r="K47" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L47" s="10">
+      <c r="L47" s="9">
         <v>70</v>
       </c>
       <c r="M47" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N47" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U47" s="9">
+      <c r="N47" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U47" s="12">
         <v>931.8</v>
       </c>
     </row>
@@ -3725,7 +3741,7 @@
       <c r="P48" s="8">
         <v>85</v>
       </c>
-      <c r="U48" s="9">
+      <c r="U48" s="12">
         <v>1129</v>
       </c>
     </row>
@@ -3745,52 +3761,52 @@
       <c r="E49" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F49" s="10">
+      <c r="F49" s="9">
         <v>600</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H49" s="10">
+      <c r="H49" s="9">
         <v>50</v>
       </c>
       <c r="I49" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J49" s="10">
+      <c r="J49" s="9">
         <v>37</v>
       </c>
       <c r="K49" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L49" s="10">
+      <c r="L49" s="9">
         <v>37</v>
       </c>
       <c r="M49" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="N49" s="10">
+      <c r="N49" s="9">
         <v>70</v>
       </c>
       <c r="O49" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P49" s="10">
+      <c r="P49" s="9">
         <v>85</v>
       </c>
       <c r="Q49" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="R49" s="10">
+      <c r="R49" s="9">
         <v>70</v>
       </c>
       <c r="S49" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="T49" s="10">
+      <c r="T49" s="9">
         <v>100</v>
       </c>
-      <c r="U49" s="9">
+      <c r="U49" s="12">
         <v>1049</v>
       </c>
     </row>
@@ -3837,7 +3853,7 @@
       <c r="N50" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U50" s="9">
+      <c r="U50" s="12">
         <v>1081.8</v>
       </c>
     </row>
@@ -3857,34 +3873,34 @@
       <c r="E51" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F51" s="10">
+      <c r="F51" s="9">
         <v>648.71</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="H51" s="10">
+      <c r="H51" s="9">
         <v>37</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="J51" s="10">
+      <c r="J51" s="9">
         <v>85</v>
       </c>
       <c r="K51" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L51" s="10">
+      <c r="L51" s="9">
         <v>70</v>
       </c>
       <c r="M51" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N51" s="10">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="U51" s="9">
+      <c r="N51" s="9">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="U51" s="12">
         <v>880.51</v>
       </c>
     </row>
@@ -3937,7 +3953,7 @@
       <c r="P52" s="8">
         <v>70</v>
       </c>
-      <c r="U52" s="9">
+      <c r="U52" s="12">
         <v>1214</v>
       </c>
     </row>
@@ -3957,40 +3973,40 @@
       <c r="E53" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F53" s="10">
+      <c r="F53" s="9">
         <v>850</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="H53" s="10">
+      <c r="H53" s="9">
         <v>50</v>
       </c>
       <c r="I53" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="J53" s="10">
+      <c r="J53" s="9">
         <v>37</v>
       </c>
       <c r="K53" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="L53" s="10">
+      <c r="L53" s="9">
         <v>37</v>
       </c>
       <c r="M53" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="N53" s="10">
+      <c r="N53" s="9">
         <v>170</v>
       </c>
       <c r="O53" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="P53" s="10">
-        <v>70</v>
-      </c>
-      <c r="U53" s="9">
+      <c r="P53" s="9">
+        <v>70</v>
+      </c>
+      <c r="U53" s="12">
         <v>1214</v>
       </c>
     </row>
@@ -4043,7 +4059,7 @@
       <c r="P54" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U54" s="9">
+      <c r="U54" s="12">
         <v>1272.75</v>
       </c>
     </row>
@@ -4063,46 +4079,46 @@
       <c r="E55" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F55" s="10">
+      <c r="F55" s="9">
         <v>500</v>
       </c>
       <c r="G55" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H55" s="10">
+      <c r="H55" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I55" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J55" s="10">
+      <c r="J55" s="9">
         <v>50</v>
       </c>
       <c r="K55" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L55" s="10">
+      <c r="L55" s="9">
         <v>70</v>
       </c>
       <c r="M55" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N55" s="10">
+      <c r="N55" s="9">
         <v>37</v>
       </c>
       <c r="O55" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="P55" s="10">
+      <c r="P55" s="9">
         <v>100</v>
       </c>
       <c r="Q55" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="R55" s="10">
+      <c r="R55" s="9">
         <v>85</v>
       </c>
-      <c r="U55" s="9">
+      <c r="U55" s="12">
         <v>881.8</v>
       </c>
     </row>
@@ -4155,7 +4171,7 @@
       <c r="P56" s="8">
         <v>-49</v>
       </c>
-      <c r="U56" s="9">
+      <c r="U56" s="12">
         <v>1181.94</v>
       </c>
     </row>
@@ -4175,46 +4191,46 @@
       <c r="E57" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F57" s="10">
+      <c r="F57" s="9">
         <v>500</v>
       </c>
       <c r="G57" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H57" s="10">
+      <c r="H57" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J57" s="10">
+      <c r="J57" s="9">
         <v>50</v>
       </c>
       <c r="K57" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L57" s="10">
+      <c r="L57" s="9">
         <v>70</v>
       </c>
       <c r="M57" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N57" s="10">
+      <c r="N57" s="9">
         <v>37</v>
       </c>
       <c r="O57" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="P57" s="10">
+      <c r="P57" s="9">
         <v>100</v>
       </c>
       <c r="Q57" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="R57" s="10">
+      <c r="R57" s="9">
         <v>85</v>
       </c>
-      <c r="U57" s="9">
+      <c r="U57" s="12">
         <v>881.8</v>
       </c>
     </row>
@@ -4255,7 +4271,7 @@
       <c r="L58" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U58" s="9">
+      <c r="U58" s="12">
         <v>823.42</v>
       </c>
     </row>
@@ -4275,40 +4291,40 @@
       <c r="E59" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F59" s="10">
+      <c r="F59" s="9">
         <v>1100</v>
       </c>
       <c r="G59" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H59" s="10">
+      <c r="H59" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I59" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J59" s="10">
+      <c r="J59" s="9">
         <v>50</v>
       </c>
       <c r="K59" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L59" s="10">
+      <c r="L59" s="9">
         <v>70</v>
       </c>
       <c r="M59" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N59" s="10">
+      <c r="N59" s="9">
         <v>37</v>
       </c>
       <c r="O59" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P59" s="10">
+      <c r="P59" s="9">
         <v>85</v>
       </c>
-      <c r="U59" s="9">
+      <c r="U59" s="12">
         <v>1381.8</v>
       </c>
     </row>
@@ -4361,7 +4377,7 @@
       <c r="P60" s="8">
         <v>170</v>
       </c>
-      <c r="U60" s="9">
+      <c r="U60" s="12">
         <v>1214</v>
       </c>
     </row>
@@ -4381,52 +4397,52 @@
       <c r="E61" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F61" s="10">
+      <c r="F61" s="9">
         <v>850</v>
       </c>
       <c r="G61" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H61" s="10">
+      <c r="H61" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I61" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J61" s="10">
+      <c r="J61" s="9">
         <v>50</v>
       </c>
       <c r="K61" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L61" s="10">
+      <c r="L61" s="9">
         <v>70</v>
       </c>
       <c r="M61" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N61" s="10">
+      <c r="N61" s="9">
         <v>37</v>
       </c>
       <c r="O61" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P61" s="10">
+      <c r="P61" s="9">
         <v>85</v>
       </c>
       <c r="Q61" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="R61" s="10">
+      <c r="R61" s="9">
         <v>141</v>
       </c>
       <c r="S61" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="T61" s="10">
+      <c r="T61" s="9">
         <v>60</v>
       </c>
-      <c r="U61" s="9">
+      <c r="U61" s="12">
         <v>1332.8</v>
       </c>
     </row>
@@ -4485,7 +4501,7 @@
       <c r="R62" s="8">
         <v>141</v>
       </c>
-      <c r="U62" s="9">
+      <c r="U62" s="12">
         <v>1357.8</v>
       </c>
     </row>
@@ -4505,40 +4521,40 @@
       <c r="E63" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F63" s="10">
+      <c r="F63" s="9">
         <v>850</v>
       </c>
       <c r="G63" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H63" s="10">
+      <c r="H63" s="9">
         <v>50</v>
       </c>
       <c r="I63" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J63" s="10">
+      <c r="J63" s="9">
         <v>37</v>
       </c>
       <c r="K63" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="L63" s="10">
+      <c r="L63" s="9">
         <v>170</v>
       </c>
       <c r="M63" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="N63" s="10">
+      <c r="N63" s="9">
         <v>37</v>
       </c>
       <c r="O63" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="P63" s="10">
-        <v>70</v>
-      </c>
-      <c r="U63" s="9">
+      <c r="P63" s="9">
+        <v>70</v>
+      </c>
+      <c r="U63" s="12">
         <v>1214</v>
       </c>
     </row>
@@ -4585,7 +4601,7 @@
       <c r="N64" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="U64" s="9">
+      <c r="U64" s="12">
         <v>1214.6300000000001</v>
       </c>
     </row>
@@ -4605,46 +4621,46 @@
       <c r="E65" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F65" s="10">
+      <c r="F65" s="9">
         <v>850</v>
       </c>
       <c r="G65" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H65" s="10">
+      <c r="H65" s="9">
         <v>39.799999999999997</v>
       </c>
       <c r="I65" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J65" s="10">
+      <c r="J65" s="9">
         <v>50</v>
       </c>
       <c r="K65" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="L65" s="10">
+      <c r="L65" s="9">
         <v>70</v>
       </c>
       <c r="M65" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N65" s="10">
+      <c r="N65" s="9">
         <v>37</v>
       </c>
       <c r="O65" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="P65" s="10">
+      <c r="P65" s="9">
         <v>141</v>
       </c>
       <c r="Q65" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="R65" s="10">
+      <c r="R65" s="9">
         <v>170</v>
       </c>
-      <c r="U65" s="9">
+      <c r="U65" s="12">
         <v>1357.8</v>
       </c>
     </row>

</xml_diff>